<commit_message>
Update extracted_data.json with additional entries and modify .gitignore to exclude virtual environment directory
</commit_message>
<xml_diff>
--- a/filtered_data.xlsx
+++ b/filtered_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="220">
   <si>
     <t>شناسه</t>
   </si>
@@ -76,6 +76,57 @@
     <t>آبادگران پاراك دشتگل</t>
   </si>
   <si>
+    <t>آتيه سازان صنعت رامهرمز</t>
+  </si>
+  <si>
+    <t>ياقوت اعتماد سرخ</t>
+  </si>
+  <si>
+    <t>قره قوم شبستر</t>
+  </si>
+  <si>
+    <t>مهندسي هوشمند آينده مانا</t>
+  </si>
+  <si>
+    <t>هيئت مذهبي محبين الحسين ع مقيم شميران</t>
+  </si>
+  <si>
+    <t>ارغوان خدمات خاورميانه</t>
+  </si>
+  <si>
+    <t>اوجان تجارت راستين</t>
+  </si>
+  <si>
+    <t>هونام پارسه البرز</t>
+  </si>
+  <si>
+    <t>كوه نگاران سهند</t>
+  </si>
+  <si>
+    <t>آركان نصب صنعت</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> بارمان اکسین رهام اروند</t>
+  </si>
+  <si>
+    <t>آران تجارت وسپار</t>
+  </si>
+  <si>
+    <t>نگين مهتاب طلاييه پارس</t>
+  </si>
+  <si>
+    <t>حامي فولاد نوين اسپادانا</t>
+  </si>
+  <si>
+    <t>درخشان ماندگار آراد</t>
+  </si>
+  <si>
+    <t>چاوش صنعت تابان</t>
+  </si>
+  <si>
+    <t>سپندار تجارت زاگرس</t>
+  </si>
+  <si>
     <t>4420591927</t>
   </si>
   <si>
@@ -169,6 +220,309 @@
     <t>1960386409</t>
   </si>
   <si>
+    <t>1960648942</t>
+  </si>
+  <si>
+    <t>5279947172</t>
+  </si>
+  <si>
+    <t>1970527528</t>
+  </si>
+  <si>
+    <t>6639577976</t>
+  </si>
+  <si>
+    <t>1900250942</t>
+  </si>
+  <si>
+    <t>1900322951</t>
+  </si>
+  <si>
+    <t>1910747505</t>
+  </si>
+  <si>
+    <t>1910802212</t>
+  </si>
+  <si>
+    <t>6000066661</t>
+  </si>
+  <si>
+    <t>3050791519</t>
+  </si>
+  <si>
+    <t>4420685077</t>
+  </si>
+  <si>
+    <t>1200172264</t>
+  </si>
+  <si>
+    <t>4421358754</t>
+  </si>
+  <si>
+    <t>4270008792</t>
+  </si>
+  <si>
+    <t>4285528691</t>
+  </si>
+  <si>
+    <t>4285580438</t>
+  </si>
+  <si>
+    <t>4270394544</t>
+  </si>
+  <si>
+    <t>4280540373</t>
+  </si>
+  <si>
+    <t>1581489536</t>
+  </si>
+  <si>
+    <t>1581491387</t>
+  </si>
+  <si>
+    <t>1583443101</t>
+  </si>
+  <si>
+    <t>5199872087</t>
+  </si>
+  <si>
+    <t>1380989353</t>
+  </si>
+  <si>
+    <t>1570341834</t>
+  </si>
+  <si>
+    <t>0451652193</t>
+  </si>
+  <si>
+    <t>0081332440</t>
+  </si>
+  <si>
+    <t>6090057843</t>
+  </si>
+  <si>
+    <t>6090086983</t>
+  </si>
+  <si>
+    <t>6090045179</t>
+  </si>
+  <si>
+    <t>6090072788</t>
+  </si>
+  <si>
+    <t>0790385597</t>
+  </si>
+  <si>
+    <t>0792301544</t>
+  </si>
+  <si>
+    <t>0062973584</t>
+  </si>
+  <si>
+    <t>0452543185</t>
+  </si>
+  <si>
+    <t>0920416829</t>
+  </si>
+  <si>
+    <t>0920451780</t>
+  </si>
+  <si>
+    <t>0923726403</t>
+  </si>
+  <si>
+    <t>0923241991</t>
+  </si>
+  <si>
+    <t>0926581929</t>
+  </si>
+  <si>
+    <t>0032263392</t>
+  </si>
+  <si>
+    <t>0067433367</t>
+  </si>
+  <si>
+    <t>0082568189</t>
+  </si>
+  <si>
+    <t>0410328588</t>
+  </si>
+  <si>
+    <t>0440341477</t>
+  </si>
+  <si>
+    <t>0453306306</t>
+  </si>
+  <si>
+    <t>0453469590</t>
+  </si>
+  <si>
+    <t>1728911702</t>
+  </si>
+  <si>
+    <t>4220224807</t>
+  </si>
+  <si>
+    <t>4220396136</t>
+  </si>
+  <si>
+    <t>2280668424</t>
+  </si>
+  <si>
+    <t>4220119231</t>
+  </si>
+  <si>
+    <t>4232224939</t>
+  </si>
+  <si>
+    <t>0312544871</t>
+  </si>
+  <si>
+    <t>1718692242</t>
+  </si>
+  <si>
+    <t>0150022077</t>
+  </si>
+  <si>
+    <t>2051299463</t>
+  </si>
+  <si>
+    <t>2130836021</t>
+  </si>
+  <si>
+    <t>2140186761</t>
+  </si>
+  <si>
+    <t>2141271568</t>
+  </si>
+  <si>
+    <t>1900255091</t>
+  </si>
+  <si>
+    <t>1900509059</t>
+  </si>
+  <si>
+    <t>1910910775</t>
+  </si>
+  <si>
+    <t>1911110845</t>
+  </si>
+  <si>
+    <t>1670831965</t>
+  </si>
+  <si>
+    <t>1671998839</t>
+  </si>
+  <si>
+    <t>6319820020</t>
+  </si>
+  <si>
+    <t>1452020231</t>
+  </si>
+  <si>
+    <t>1465789804</t>
+  </si>
+  <si>
+    <t>4660262103</t>
+  </si>
+  <si>
+    <t>4660333450</t>
+  </si>
+  <si>
+    <t>4660482839</t>
+  </si>
+  <si>
+    <t>4660221415</t>
+  </si>
+  <si>
+    <t>4660505472</t>
+  </si>
+  <si>
+    <t>4132113760</t>
+  </si>
+  <si>
+    <t>2580193286</t>
+  </si>
+  <si>
+    <t>1960535544</t>
+  </si>
+  <si>
+    <t>1960587961</t>
+  </si>
+  <si>
+    <t>5559447366</t>
+  </si>
+  <si>
+    <t>1960441590</t>
+  </si>
+  <si>
+    <t>1960456660</t>
+  </si>
+  <si>
+    <t>0829438211</t>
+  </si>
+  <si>
+    <t>0921402333</t>
+  </si>
+  <si>
+    <t>0945454503</t>
+  </si>
+  <si>
+    <t>0938982397</t>
+  </si>
+  <si>
+    <t>0939722615</t>
+  </si>
+  <si>
+    <t>1111793689</t>
+  </si>
+  <si>
+    <t>1249958180</t>
+  </si>
+  <si>
+    <t>2296231871</t>
+  </si>
+  <si>
+    <t>1272662721</t>
+  </si>
+  <si>
+    <t>1289075441</t>
+  </si>
+  <si>
+    <t>4810132511</t>
+  </si>
+  <si>
+    <t>4810196658</t>
+  </si>
+  <si>
+    <t>4810270947</t>
+  </si>
+  <si>
+    <t>1900207907</t>
+  </si>
+  <si>
+    <t>1900456893</t>
+  </si>
+  <si>
+    <t>0010866787</t>
+  </si>
+  <si>
+    <t>0013610546</t>
+  </si>
+  <si>
+    <t>0310882230</t>
+  </si>
+  <si>
+    <t>1271405849</t>
+  </si>
+  <si>
+    <t>1276407750</t>
+  </si>
+  <si>
+    <t>4622161036</t>
+  </si>
+  <si>
     <t>مدیرعامل</t>
   </si>
   <si>
@@ -187,6 +541,9 @@
     <t>عضو هیئت مدیره</t>
   </si>
   <si>
+    <t>نامشخص</t>
+  </si>
+  <si>
     <t>2025-05-01 10:55:05</t>
   </si>
   <si>
@@ -239,6 +596,84 @@
   </si>
   <si>
     <t>2025-05-01 11:28:21</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:12:19</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:12:21</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:00</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:02</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:04</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:10</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:11</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:14</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:16</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:17</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:19</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:20</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:22</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:24</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:30</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:31</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:32</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:34</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:35</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:37</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:39</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:41</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:42</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:44</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:49</t>
+  </si>
+  <si>
+    <t>2025-05-03 12:14:51</t>
   </si>
 </sst>
 </file>
@@ -596,7 +1031,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -624,13 +1059,13 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -641,13 +1076,13 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -658,13 +1093,13 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -675,13 +1110,13 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -692,13 +1127,13 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -709,13 +1144,13 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>172</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -726,13 +1161,13 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>173</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -743,13 +1178,13 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -760,13 +1195,13 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>174</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -777,13 +1212,13 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -794,13 +1229,13 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -811,13 +1246,13 @@
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E13" t="s">
-        <v>61</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -828,13 +1263,13 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -845,13 +1280,13 @@
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E15" t="s">
-        <v>63</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -862,13 +1297,13 @@
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -879,13 +1314,13 @@
         <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="D17" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E17" t="s">
-        <v>65</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -896,13 +1331,13 @@
         <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="D18" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E18" t="s">
-        <v>66</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -913,13 +1348,13 @@
         <v>15</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -930,13 +1365,13 @@
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="D20" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E20" t="s">
-        <v>68</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -947,13 +1382,13 @@
         <v>17</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="D21" t="s">
-        <v>51</v>
+        <v>169</v>
       </c>
       <c r="E21" t="s">
-        <v>69</v>
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -964,13 +1399,13 @@
         <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="D22" t="s">
-        <v>54</v>
+        <v>172</v>
       </c>
       <c r="E22" t="s">
-        <v>70</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -981,13 +1416,13 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="D23" t="s">
-        <v>55</v>
+        <v>173</v>
       </c>
       <c r="E23" t="s">
-        <v>70</v>
+        <v>189</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -998,13 +1433,13 @@
         <v>18</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="D24" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="E24" t="s">
-        <v>71</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1015,13 +1450,13 @@
         <v>18</v>
       </c>
       <c r="C25" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="D25" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="E25" t="s">
-        <v>71</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1032,13 +1467,13 @@
         <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>172</v>
       </c>
       <c r="E26" t="s">
-        <v>71</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1049,13 +1484,13 @@
         <v>8</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="D27" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="E27" t="s">
-        <v>72</v>
+        <v>191</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1066,13 +1501,13 @@
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="D28" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1083,13 +1518,13 @@
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="D29" t="s">
-        <v>56</v>
+        <v>174</v>
       </c>
       <c r="E29" t="s">
-        <v>73</v>
+        <v>192</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1100,13 +1535,13 @@
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="D30" t="s">
-        <v>55</v>
+        <v>173</v>
       </c>
       <c r="E30" t="s">
-        <v>73</v>
+        <v>192</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -1117,13 +1552,13 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>54</v>
+        <v>172</v>
       </c>
       <c r="E31" t="s">
-        <v>73</v>
+        <v>192</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -1134,13 +1569,1798 @@
         <v>19</v>
       </c>
       <c r="C32" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" t="s">
+        <v>170</v>
+      </c>
+      <c r="E32" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33" t="s">
+        <v>171</v>
+      </c>
+      <c r="E33" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" t="s">
+        <v>69</v>
+      </c>
+      <c r="D34" t="s">
+        <v>174</v>
+      </c>
+      <c r="E34" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D35" t="s">
+        <v>173</v>
+      </c>
+      <c r="E35" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" t="s">
+        <v>172</v>
+      </c>
+      <c r="E36" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" t="s">
+        <v>72</v>
+      </c>
+      <c r="D37" t="s">
+        <v>174</v>
+      </c>
+      <c r="E37" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" t="s">
+        <v>73</v>
+      </c>
+      <c r="D38" t="s">
+        <v>170</v>
+      </c>
+      <c r="E38" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" t="s">
+        <v>74</v>
+      </c>
+      <c r="D39" t="s">
+        <v>171</v>
+      </c>
+      <c r="E39" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" t="s">
+        <v>172</v>
+      </c>
+      <c r="E40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>20</v>
+      </c>
+      <c r="C41" t="s">
+        <v>76</v>
+      </c>
+      <c r="D41" t="s">
+        <v>173</v>
+      </c>
+      <c r="E41" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D42" t="s">
+        <v>171</v>
+      </c>
+      <c r="E42" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" t="s">
+        <v>78</v>
+      </c>
+      <c r="D43" t="s">
+        <v>170</v>
+      </c>
+      <c r="E43" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" t="s">
+        <v>79</v>
+      </c>
+      <c r="D44" t="s">
+        <v>172</v>
+      </c>
+      <c r="E44" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" t="s">
+        <v>173</v>
+      </c>
+      <c r="E45" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" t="s">
+        <v>81</v>
+      </c>
+      <c r="D46" t="s">
+        <v>174</v>
+      </c>
+      <c r="E46" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" t="s">
+        <v>82</v>
+      </c>
+      <c r="D47" t="s">
+        <v>174</v>
+      </c>
+      <c r="E47" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" t="s">
+        <v>83</v>
+      </c>
+      <c r="D48" t="s">
+        <v>174</v>
+      </c>
+      <c r="E48" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" t="s">
+        <v>84</v>
+      </c>
+      <c r="D49" t="s">
+        <v>173</v>
+      </c>
+      <c r="E49" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>21</v>
+      </c>
+      <c r="C50" t="s">
+        <v>85</v>
+      </c>
+      <c r="D50" t="s">
+        <v>172</v>
+      </c>
+      <c r="E50" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51">
         <v>50</v>
       </c>
-      <c r="D32" t="s">
+      <c r="B51" t="s">
+        <v>22</v>
+      </c>
+      <c r="C51" t="s">
+        <v>86</v>
+      </c>
+      <c r="D51" t="s">
+        <v>174</v>
+      </c>
+      <c r="E51" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>22</v>
+      </c>
+      <c r="C52" t="s">
+        <v>87</v>
+      </c>
+      <c r="D52" t="s">
+        <v>174</v>
+      </c>
+      <c r="E52" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53">
         <v>52</v>
       </c>
-      <c r="E32" t="s">
+      <c r="B53" t="s">
+        <v>22</v>
+      </c>
+      <c r="C53" t="s">
+        <v>88</v>
+      </c>
+      <c r="D53" t="s">
+        <v>174</v>
+      </c>
+      <c r="E53" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>22</v>
+      </c>
+      <c r="C54" t="s">
+        <v>89</v>
+      </c>
+      <c r="D54" t="s">
+        <v>174</v>
+      </c>
+      <c r="E54" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>22</v>
+      </c>
+      <c r="C55" t="s">
+        <v>90</v>
+      </c>
+      <c r="D55" t="s">
+        <v>173</v>
+      </c>
+      <c r="E55" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>22</v>
+      </c>
+      <c r="C56" t="s">
+        <v>91</v>
+      </c>
+      <c r="D56" t="s">
+        <v>172</v>
+      </c>
+      <c r="E56" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" t="s">
+        <v>92</v>
+      </c>
+      <c r="D57" t="s">
+        <v>174</v>
+      </c>
+      <c r="E57" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>13</v>
+      </c>
+      <c r="C58" t="s">
+        <v>93</v>
+      </c>
+      <c r="D58" t="s">
+        <v>170</v>
+      </c>
+      <c r="E58" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" t="s">
+        <v>94</v>
+      </c>
+      <c r="D59" t="s">
+        <v>171</v>
+      </c>
+      <c r="E59" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60" t="s">
+        <v>95</v>
+      </c>
+      <c r="D60" t="s">
+        <v>170</v>
+      </c>
+      <c r="E60" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" t="s">
+        <v>96</v>
+      </c>
+      <c r="D61" t="s">
+        <v>173</v>
+      </c>
+      <c r="E61" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62" t="s">
+        <v>97</v>
+      </c>
+      <c r="D62" t="s">
+        <v>172</v>
+      </c>
+      <c r="E62" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>15</v>
+      </c>
+      <c r="C63" t="s">
+        <v>98</v>
+      </c>
+      <c r="D63" t="s">
+        <v>170</v>
+      </c>
+      <c r="E63" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>15</v>
+      </c>
+      <c r="C64" t="s">
+        <v>99</v>
+      </c>
+      <c r="D64" t="s">
+        <v>174</v>
+      </c>
+      <c r="E64" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>15</v>
+      </c>
+      <c r="C65" t="s">
+        <v>100</v>
+      </c>
+      <c r="D65" t="s">
+        <v>172</v>
+      </c>
+      <c r="E65" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>15</v>
+      </c>
+      <c r="C66" t="s">
+        <v>101</v>
+      </c>
+      <c r="D66" t="s">
+        <v>173</v>
+      </c>
+      <c r="E66" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>23</v>
+      </c>
+      <c r="C67" t="s">
+        <v>102</v>
+      </c>
+      <c r="D67" t="s">
+        <v>174</v>
+      </c>
+      <c r="E67" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>23</v>
+      </c>
+      <c r="C68" t="s">
+        <v>103</v>
+      </c>
+      <c r="D68" t="s">
+        <v>170</v>
+      </c>
+      <c r="E68" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>23</v>
+      </c>
+      <c r="C69" t="s">
+        <v>104</v>
+      </c>
+      <c r="D69" t="s">
+        <v>171</v>
+      </c>
+      <c r="E69" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>23</v>
+      </c>
+      <c r="C70" t="s">
+        <v>105</v>
+      </c>
+      <c r="D70" t="s">
+        <v>172</v>
+      </c>
+      <c r="E70" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>23</v>
+      </c>
+      <c r="C71" t="s">
+        <v>106</v>
+      </c>
+      <c r="D71" t="s">
+        <v>173</v>
+      </c>
+      <c r="E71" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>24</v>
+      </c>
+      <c r="C72" t="s">
+        <v>107</v>
+      </c>
+      <c r="D72" t="s">
+        <v>174</v>
+      </c>
+      <c r="E72" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>24</v>
+      </c>
+      <c r="C73" t="s">
+        <v>108</v>
+      </c>
+      <c r="D73" t="s">
+        <v>174</v>
+      </c>
+      <c r="E73" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>24</v>
+      </c>
+      <c r="C74" t="s">
+        <v>109</v>
+      </c>
+      <c r="D74" t="s">
+        <v>174</v>
+      </c>
+      <c r="E74" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75">
         <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>24</v>
+      </c>
+      <c r="C75" t="s">
+        <v>110</v>
+      </c>
+      <c r="D75" t="s">
+        <v>175</v>
+      </c>
+      <c r="E75" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>24</v>
+      </c>
+      <c r="C76" t="s">
+        <v>111</v>
+      </c>
+      <c r="D76" t="s">
+        <v>175</v>
+      </c>
+      <c r="E76" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>24</v>
+      </c>
+      <c r="C77" t="s">
+        <v>112</v>
+      </c>
+      <c r="D77" t="s">
+        <v>174</v>
+      </c>
+      <c r="E77" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>24</v>
+      </c>
+      <c r="C78" t="s">
+        <v>113</v>
+      </c>
+      <c r="D78" t="s">
+        <v>174</v>
+      </c>
+      <c r="E78" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>24</v>
+      </c>
+      <c r="C79" t="s">
+        <v>114</v>
+      </c>
+      <c r="D79" t="s">
+        <v>174</v>
+      </c>
+      <c r="E79" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>25</v>
+      </c>
+      <c r="C80" t="s">
+        <v>115</v>
+      </c>
+      <c r="D80" t="s">
+        <v>174</v>
+      </c>
+      <c r="E80" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>25</v>
+      </c>
+      <c r="C81" t="s">
+        <v>116</v>
+      </c>
+      <c r="D81" t="s">
+        <v>171</v>
+      </c>
+      <c r="E81" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>25</v>
+      </c>
+      <c r="C82" t="s">
+        <v>55</v>
+      </c>
+      <c r="D82" t="s">
+        <v>170</v>
+      </c>
+      <c r="E82" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>25</v>
+      </c>
+      <c r="C83" t="s">
+        <v>117</v>
+      </c>
+      <c r="D83" t="s">
+        <v>173</v>
+      </c>
+      <c r="E83" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>25</v>
+      </c>
+      <c r="C84" t="s">
+        <v>118</v>
+      </c>
+      <c r="D84" t="s">
+        <v>172</v>
+      </c>
+      <c r="E84" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>16</v>
+      </c>
+      <c r="C85" t="s">
+        <v>115</v>
+      </c>
+      <c r="D85" t="s">
+        <v>170</v>
+      </c>
+      <c r="E85" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>16</v>
+      </c>
+      <c r="C86" t="s">
+        <v>119</v>
+      </c>
+      <c r="D86" t="s">
+        <v>171</v>
+      </c>
+      <c r="E86" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>16</v>
+      </c>
+      <c r="C87" t="s">
+        <v>117</v>
+      </c>
+      <c r="D87" t="s">
+        <v>173</v>
+      </c>
+      <c r="E87" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>16</v>
+      </c>
+      <c r="C88" t="s">
+        <v>118</v>
+      </c>
+      <c r="D88" t="s">
+        <v>172</v>
+      </c>
+      <c r="E88" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>26</v>
+      </c>
+      <c r="C89" t="s">
+        <v>120</v>
+      </c>
+      <c r="D89" t="s">
+        <v>170</v>
+      </c>
+      <c r="E89" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>26</v>
+      </c>
+      <c r="C90" t="s">
+        <v>121</v>
+      </c>
+      <c r="D90" t="s">
+        <v>174</v>
+      </c>
+      <c r="E90" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>27</v>
+      </c>
+      <c r="C91" t="s">
+        <v>122</v>
+      </c>
+      <c r="D91" t="s">
+        <v>174</v>
+      </c>
+      <c r="E91" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C92" t="s">
+        <v>123</v>
+      </c>
+      <c r="D92" t="s">
+        <v>169</v>
+      </c>
+      <c r="E92" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C93" t="s">
+        <v>124</v>
+      </c>
+      <c r="D93" t="s">
+        <v>174</v>
+      </c>
+      <c r="E93" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>27</v>
+      </c>
+      <c r="C94" t="s">
+        <v>125</v>
+      </c>
+      <c r="D94" t="s">
+        <v>172</v>
+      </c>
+      <c r="E94" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>27</v>
+      </c>
+      <c r="C95" t="s">
+        <v>126</v>
+      </c>
+      <c r="D95" t="s">
+        <v>173</v>
+      </c>
+      <c r="E95" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>17</v>
+      </c>
+      <c r="C96" t="s">
+        <v>127</v>
+      </c>
+      <c r="D96" t="s">
+        <v>171</v>
+      </c>
+      <c r="E96" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>17</v>
+      </c>
+      <c r="C97" t="s">
+        <v>128</v>
+      </c>
+      <c r="D97" t="s">
+        <v>170</v>
+      </c>
+      <c r="E97" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>17</v>
+      </c>
+      <c r="C98" t="s">
+        <v>129</v>
+      </c>
+      <c r="D98" t="s">
+        <v>172</v>
+      </c>
+      <c r="E98" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>17</v>
+      </c>
+      <c r="C99" t="s">
+        <v>130</v>
+      </c>
+      <c r="D99" t="s">
+        <v>173</v>
+      </c>
+      <c r="E99" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>28</v>
+      </c>
+      <c r="C100" t="s">
+        <v>131</v>
+      </c>
+      <c r="D100" t="s">
+        <v>170</v>
+      </c>
+      <c r="E100" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>28</v>
+      </c>
+      <c r="C101" t="s">
+        <v>132</v>
+      </c>
+      <c r="D101" t="s">
+        <v>171</v>
+      </c>
+      <c r="E101" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>28</v>
+      </c>
+      <c r="C102" t="s">
+        <v>133</v>
+      </c>
+      <c r="D102" t="s">
+        <v>169</v>
+      </c>
+      <c r="E102" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>28</v>
+      </c>
+      <c r="C103" t="s">
+        <v>134</v>
+      </c>
+      <c r="D103" t="s">
+        <v>173</v>
+      </c>
+      <c r="E103" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>28</v>
+      </c>
+      <c r="C104" t="s">
+        <v>135</v>
+      </c>
+      <c r="D104" t="s">
+        <v>172</v>
+      </c>
+      <c r="E104" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>29</v>
+      </c>
+      <c r="C105" t="s">
+        <v>136</v>
+      </c>
+      <c r="D105" t="s">
+        <v>170</v>
+      </c>
+      <c r="E105" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>29</v>
+      </c>
+      <c r="C106" t="s">
+        <v>137</v>
+      </c>
+      <c r="D106" t="s">
+        <v>171</v>
+      </c>
+      <c r="E106" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>29</v>
+      </c>
+      <c r="C107" t="s">
+        <v>138</v>
+      </c>
+      <c r="D107" t="s">
+        <v>169</v>
+      </c>
+      <c r="E107" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="s">
+        <v>29</v>
+      </c>
+      <c r="C108" t="s">
+        <v>139</v>
+      </c>
+      <c r="D108" t="s">
+        <v>173</v>
+      </c>
+      <c r="E108" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="s">
+        <v>29</v>
+      </c>
+      <c r="C109" t="s">
+        <v>140</v>
+      </c>
+      <c r="D109" t="s">
+        <v>172</v>
+      </c>
+      <c r="E109" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="s">
+        <v>30</v>
+      </c>
+      <c r="C110" t="s">
+        <v>141</v>
+      </c>
+      <c r="D110" t="s">
+        <v>172</v>
+      </c>
+      <c r="E110" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>30</v>
+      </c>
+      <c r="C111" t="s">
+        <v>142</v>
+      </c>
+      <c r="D111" t="s">
+        <v>173</v>
+      </c>
+      <c r="E111" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>31</v>
+      </c>
+      <c r="C112" t="s">
+        <v>143</v>
+      </c>
+      <c r="D112" t="s">
+        <v>170</v>
+      </c>
+      <c r="E112" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>31</v>
+      </c>
+      <c r="C113" t="s">
+        <v>144</v>
+      </c>
+      <c r="D113" t="s">
+        <v>171</v>
+      </c>
+      <c r="E113" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="s">
+        <v>31</v>
+      </c>
+      <c r="C114" t="s">
+        <v>145</v>
+      </c>
+      <c r="D114" t="s">
+        <v>169</v>
+      </c>
+      <c r="E114" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>31</v>
+      </c>
+      <c r="C115" t="s">
+        <v>146</v>
+      </c>
+      <c r="D115" t="s">
+        <v>172</v>
+      </c>
+      <c r="E115" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>31</v>
+      </c>
+      <c r="C116" t="s">
+        <v>147</v>
+      </c>
+      <c r="D116" t="s">
+        <v>173</v>
+      </c>
+      <c r="E116" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>32</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117" t="s">
+        <v>171</v>
+      </c>
+      <c r="E117" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>32</v>
+      </c>
+      <c r="C118" t="s">
+        <v>149</v>
+      </c>
+      <c r="D118" t="s">
+        <v>169</v>
+      </c>
+      <c r="E118" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>32</v>
+      </c>
+      <c r="C119" t="s">
+        <v>150</v>
+      </c>
+      <c r="D119" t="s">
+        <v>170</v>
+      </c>
+      <c r="E119" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="s">
+        <v>32</v>
+      </c>
+      <c r="C120" t="s">
+        <v>151</v>
+      </c>
+      <c r="D120" t="s">
+        <v>173</v>
+      </c>
+      <c r="E120" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>32</v>
+      </c>
+      <c r="C121" t="s">
+        <v>152</v>
+      </c>
+      <c r="D121" t="s">
+        <v>172</v>
+      </c>
+      <c r="E121" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="s">
+        <v>33</v>
+      </c>
+      <c r="C122" t="s">
+        <v>153</v>
+      </c>
+      <c r="D122" t="s">
+        <v>170</v>
+      </c>
+      <c r="E122" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="s">
+        <v>33</v>
+      </c>
+      <c r="C123" t="s">
+        <v>154</v>
+      </c>
+      <c r="D123" t="s">
+        <v>169</v>
+      </c>
+      <c r="E123" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="s">
+        <v>33</v>
+      </c>
+      <c r="C124" t="s">
+        <v>155</v>
+      </c>
+      <c r="D124" t="s">
+        <v>174</v>
+      </c>
+      <c r="E124" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="s">
+        <v>33</v>
+      </c>
+      <c r="C125" t="s">
+        <v>156</v>
+      </c>
+      <c r="D125" t="s">
+        <v>172</v>
+      </c>
+      <c r="E125" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="s">
+        <v>33</v>
+      </c>
+      <c r="C126" t="s">
+        <v>157</v>
+      </c>
+      <c r="D126" t="s">
+        <v>173</v>
+      </c>
+      <c r="E126" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
+        <v>34</v>
+      </c>
+      <c r="C127" t="s">
+        <v>158</v>
+      </c>
+      <c r="D127" t="s">
+        <v>170</v>
+      </c>
+      <c r="E127" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="s">
+        <v>34</v>
+      </c>
+      <c r="C128" t="s">
+        <v>159</v>
+      </c>
+      <c r="D128" t="s">
+        <v>169</v>
+      </c>
+      <c r="E128" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="s">
+        <v>34</v>
+      </c>
+      <c r="C129" t="s">
+        <v>160</v>
+      </c>
+      <c r="D129" t="s">
+        <v>171</v>
+      </c>
+      <c r="E129" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="s">
+        <v>34</v>
+      </c>
+      <c r="C130" t="s">
+        <v>161</v>
+      </c>
+      <c r="D130" t="s">
+        <v>172</v>
+      </c>
+      <c r="E130" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
+        <v>34</v>
+      </c>
+      <c r="C131" t="s">
+        <v>162</v>
+      </c>
+      <c r="D131" t="s">
+        <v>173</v>
+      </c>
+      <c r="E131" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
+        <v>35</v>
+      </c>
+      <c r="C132" t="s">
+        <v>163</v>
+      </c>
+      <c r="D132" t="s">
+        <v>174</v>
+      </c>
+      <c r="E132" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>35</v>
+      </c>
+      <c r="C133" t="s">
+        <v>164</v>
+      </c>
+      <c r="D133" t="s">
+        <v>171</v>
+      </c>
+      <c r="E133" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
+        <v>35</v>
+      </c>
+      <c r="C134" t="s">
+        <v>165</v>
+      </c>
+      <c r="D134" t="s">
+        <v>174</v>
+      </c>
+      <c r="E134" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
+        <v>36</v>
+      </c>
+      <c r="C135" t="s">
+        <v>166</v>
+      </c>
+      <c r="D135" t="s">
+        <v>171</v>
+      </c>
+      <c r="E135" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>36</v>
+      </c>
+      <c r="C136" t="s">
+        <v>167</v>
+      </c>
+      <c r="D136" t="s">
+        <v>170</v>
+      </c>
+      <c r="E136" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>36</v>
+      </c>
+      <c r="C137" t="s">
+        <v>168</v>
+      </c>
+      <c r="D137" t="s">
+        <v>169</v>
+      </c>
+      <c r="E137" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>